<commit_message>
slight improves to select unit and fed no
</commit_message>
<xml_diff>
--- a/Austerlitz/Turns/350FJan1808.xlsx
+++ b/Austerlitz/Turns/350FJan1808.xlsx
@@ -4272,12 +4272,12 @@
       </c>
       <c r="B157" s="10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C157" s="10" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>61</t>
         </is>
       </c>
       <c r="D157" s="4"/>
@@ -4338,12 +4338,12 @@
       </c>
       <c r="B158" s="10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4009</t>
         </is>
       </c>
       <c r="C158" s="10" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>61</t>
         </is>
       </c>
       <c r="D158" s="4"/>
@@ -4402,8 +4402,16 @@
       <c r="A159" s="4">
         <v>4</v>
       </c>
-      <c r="B159" s="10"/>
-      <c r="C159" s="10"/>
+      <c r="B159" s="10" t="inlineStr">
+        <is>
+          <t>4010</t>
+        </is>
+      </c>
+      <c r="C159" s="10" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="D159" s="4"/>
       <c r="E159" s="4"/>
       <c r="F159" s="4"/>
@@ -4460,8 +4468,16 @@
       <c r="A160" s="4">
         <v>5</v>
       </c>
-      <c r="B160" s="10"/>
-      <c r="C160" s="10"/>
+      <c r="B160" s="10" t="inlineStr">
+        <is>
+          <t>4011</t>
+        </is>
+      </c>
+      <c r="C160" s="10" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="D160" s="4"/>
       <c r="E160" s="4"/>
       <c r="F160" s="4"/>
@@ -4518,8 +4534,16 @@
       <c r="A161" s="4">
         <v>6</v>
       </c>
-      <c r="B161" s="10"/>
-      <c r="C161" s="10"/>
+      <c r="B161" s="10" t="inlineStr">
+        <is>
+          <t>4012</t>
+        </is>
+      </c>
+      <c r="C161" s="10" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="D161" s="4"/>
       <c r="E161" s="4"/>
       <c r="F161" s="4"/>
@@ -4576,8 +4600,16 @@
       <c r="A162" s="4">
         <v>7</v>
       </c>
-      <c r="B162" s="10"/>
-      <c r="C162" s="10"/>
+      <c r="B162" s="10" t="inlineStr">
+        <is>
+          <t>4013</t>
+        </is>
+      </c>
+      <c r="C162" s="10" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="D162" s="4"/>
       <c r="E162" s="4"/>
       <c r="F162" s="4"/>
@@ -4634,8 +4666,16 @@
       <c r="A163" s="4">
         <v>8</v>
       </c>
-      <c r="B163" s="10"/>
-      <c r="C163" s="10"/>
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>4014</t>
+        </is>
+      </c>
+      <c r="C163" s="10" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="D163" s="4"/>
       <c r="E163" s="4"/>
       <c r="F163" s="4"/>
@@ -4692,8 +4732,16 @@
       <c r="A164" s="4">
         <v>9</v>
       </c>
-      <c r="B164" s="10"/>
-      <c r="C164" s="10"/>
+      <c r="B164" s="10" t="inlineStr">
+        <is>
+          <t>1090</t>
+        </is>
+      </c>
+      <c r="C164" s="10" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="D164" s="4"/>
       <c r="E164" s="22"/>
       <c r="F164" s="22"/>
@@ -4750,8 +4798,16 @@
       <c r="A165" s="4">
         <v>10</v>
       </c>
-      <c r="B165" s="10"/>
-      <c r="C165" s="10"/>
+      <c r="B165" s="10" t="inlineStr">
+        <is>
+          <t>4017</t>
+        </is>
+      </c>
+      <c r="C165" s="10" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="D165" s="4"/>
       <c r="E165" s="22"/>
       <c r="F165" s="22"/>
@@ -4808,8 +4864,16 @@
       <c r="A166" s="4">
         <v>11</v>
       </c>
-      <c r="B166" s="17"/>
-      <c r="C166" s="10"/>
+      <c r="B166" s="17" t="inlineStr">
+        <is>
+          <t>4018</t>
+        </is>
+      </c>
+      <c r="C166" s="10" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="D166" s="4"/>
       <c r="E166" s="22"/>
       <c r="F166" s="22"/>
@@ -4866,8 +4930,16 @@
       <c r="A167" s="4">
         <v>12</v>
       </c>
-      <c r="B167" s="10"/>
-      <c r="C167" s="17"/>
+      <c r="B167" s="10" t="inlineStr">
+        <is>
+          <t>4016</t>
+        </is>
+      </c>
+      <c r="C167" s="17" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="D167" s="4"/>
       <c r="E167" s="22"/>
       <c r="F167" s="22"/>
@@ -4924,8 +4996,16 @@
       <c r="A168" s="4">
         <v>13</v>
       </c>
-      <c r="B168" s="10"/>
-      <c r="C168" s="10"/>
+      <c r="B168" s="10" t="inlineStr">
+        <is>
+          <t>4015</t>
+        </is>
+      </c>
+      <c r="C168" s="10" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="D168" s="4"/>
       <c r="E168" s="22"/>
       <c r="F168" s="22"/>

</xml_diff>